<commit_message>
Tufts electricity calibration corrections
</commit_message>
<xml_diff>
--- a/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
+++ b/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/BCRbQ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC1D879-A8BD-6940-95F8-60FD319F4D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D60CC50-7280-3E47-BB25-89FDB285D75B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>BCRbQ BAU Capacity Retirements before Quantization</t>
   </si>
@@ -143,6 +143,27 @@
   </si>
   <si>
     <t>GW to MW</t>
+  </si>
+  <si>
+    <t>coal</t>
+  </si>
+  <si>
+    <t>Capacity retirements (MW)</t>
+  </si>
+  <si>
+    <t>2020-2025</t>
+  </si>
+  <si>
+    <t>2026-2030</t>
+  </si>
+  <si>
+    <t>2031-2035</t>
+  </si>
+  <si>
+    <t>2036-2040</t>
+  </si>
+  <si>
+    <t>2041-2045</t>
   </si>
 </sst>
 </file>
@@ -288,6 +309,50 @@
     </xdr:pic>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5E7F1FC-B333-8796-9C14-49992B89A1F1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9017000" y="6680200"/>
+          <a:ext cx="9867900" cy="5905500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1803,103 +1868,79 @@
         <v>24</v>
       </c>
       <c r="AC3" s="5">
-        <f t="shared" ref="AC3:AK3" si="0">TREND($AB$7:$AC$7,$AB$6:$AC$6,AC2)</f>
-        <v>22.100000000000364</v>
-      </c>
-      <c r="AD3">
-        <f t="shared" si="0"/>
-        <v>20.200000000000273</v>
-      </c>
-      <c r="AE3">
-        <f t="shared" si="0"/>
-        <v>18.300000000000182</v>
-      </c>
-      <c r="AF3">
-        <f t="shared" si="0"/>
-        <v>16.400000000000091</v>
-      </c>
-      <c r="AG3">
-        <f t="shared" si="0"/>
-        <v>14.5</v>
-      </c>
-      <c r="AH3">
-        <f t="shared" si="0"/>
-        <v>12.600000000000364</v>
-      </c>
-      <c r="AI3">
-        <f t="shared" si="0"/>
-        <v>10.700000000000273</v>
-      </c>
-      <c r="AJ3">
-        <f t="shared" si="0"/>
-        <v>8.8000000000001819</v>
-      </c>
-      <c r="AK3">
-        <f t="shared" si="0"/>
-        <v>6.9000000000000909</v>
+        <v>0</v>
+      </c>
+      <c r="AD3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AJ3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AK3" s="5">
+        <v>0</v>
       </c>
       <c r="AL3" s="5">
         <v>5</v>
       </c>
       <c r="AM3" s="5">
-        <f>(AL3+AL3*$AI$5)</f>
-        <v>3.6231884057970536</v>
+        <v>0</v>
       </c>
       <c r="AN3" s="5">
-        <f t="shared" ref="AN3:BA3" si="1">(AM3+AM3*$AI$5)</f>
-        <v>2.6254988447804388</v>
+        <v>0</v>
       </c>
       <c r="AO3" s="5">
-        <f t="shared" si="1"/>
-        <v>1.9025353947684089</v>
+        <v>0</v>
       </c>
       <c r="AP3" s="5">
-        <f t="shared" si="1"/>
-        <v>1.378648836788684</v>
+        <v>0</v>
       </c>
       <c r="AQ3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.99902089622367085</v>
+        <v>0</v>
       </c>
       <c r="AR3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.72392818566931716</v>
+        <v>0</v>
       </c>
       <c r="AS3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.5245856417893533</v>
+        <v>0</v>
       </c>
       <c r="AT3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.38013452303575823</v>
+        <v>0</v>
       </c>
       <c r="AU3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.27545979930127046</v>
+        <v>0</v>
       </c>
       <c r="AV3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.19960855021830931</v>
+        <v>0</v>
       </c>
       <c r="AW3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.14464387696978745</v>
+        <v>0</v>
       </c>
       <c r="AX3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.10481440360129388</v>
+        <v>0</v>
       </c>
       <c r="AY3" s="5">
-        <f t="shared" si="1"/>
-        <v>7.595246637774819E-2</v>
+        <v>0</v>
       </c>
       <c r="AZ3" s="5">
-        <f t="shared" si="1"/>
-        <v>5.5038019114309555E-2</v>
+        <v>0</v>
       </c>
       <c r="BA3" s="5">
-        <f t="shared" si="1"/>
-        <v>3.9882622546600605E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1916,9 +1957,9 @@
       <c r="AH5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AI5">
+      <c r="AI5" t="e">
         <f>(AL3-AK3)/AK3</f>
-        <v>-0.27536231884058926</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1943,212 +1984,212 @@
         <v>12</v>
       </c>
       <c r="B9" s="10">
-        <f t="shared" ref="B9:AB9" si="2">B3*$B$5</f>
+        <f t="shared" ref="B9:AB9" si="0">B3*$B$5</f>
         <v>0</v>
       </c>
       <c r="C9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="E9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>1100</v>
       </c>
       <c r="I9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>1000</v>
       </c>
       <c r="N9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="T9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="U9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="W9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>10000</v>
       </c>
       <c r="X9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Y9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Z9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AA9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AB9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>24000</v>
       </c>
       <c r="AC9" s="10">
-        <f t="shared" ref="AC9:BA9" si="3">AC3*$B$5</f>
-        <v>22100.000000000364</v>
+        <f t="shared" ref="AC9:BA9" si="1">AC3*$B$5</f>
+        <v>0</v>
       </c>
       <c r="AD9" s="10">
-        <f t="shared" si="3"/>
-        <v>20200.000000000273</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AE9" s="10">
-        <f t="shared" si="3"/>
-        <v>18300.000000000182</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AF9" s="10">
-        <f t="shared" si="3"/>
-        <v>16400.000000000091</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AG9" s="10">
-        <f t="shared" si="3"/>
-        <v>14500</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AH9" s="10">
-        <f t="shared" si="3"/>
-        <v>12600.000000000364</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AI9" s="10">
-        <f t="shared" si="3"/>
-        <v>10700.000000000273</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AJ9" s="10">
-        <f t="shared" si="3"/>
-        <v>8800.0000000001819</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AK9" s="10">
-        <f t="shared" si="3"/>
-        <v>6900.0000000000909</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AL9" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>5000</v>
       </c>
       <c r="AM9" s="10">
-        <f t="shared" si="3"/>
-        <v>3623.1884057970537</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AN9" s="10">
-        <f t="shared" si="3"/>
-        <v>2625.498844780439</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AO9" s="10">
-        <f t="shared" si="3"/>
-        <v>1902.5353947684089</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AP9" s="10">
-        <f t="shared" si="3"/>
-        <v>1378.6488367886841</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AQ9" s="10">
-        <f t="shared" si="3"/>
-        <v>999.02089622367089</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AR9" s="10">
-        <f t="shared" si="3"/>
-        <v>723.92818566931714</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AS9" s="10">
-        <f t="shared" si="3"/>
-        <v>524.5856417893533</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AT9" s="10">
-        <f t="shared" si="3"/>
-        <v>380.13452303575821</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AU9" s="10">
-        <f t="shared" si="3"/>
-        <v>275.45979930127044</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AV9" s="10">
-        <f t="shared" si="3"/>
-        <v>199.60855021830932</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AW9" s="10">
-        <f t="shared" si="3"/>
-        <v>144.64387696978744</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AX9" s="10">
-        <f t="shared" si="3"/>
-        <v>104.81440360129388</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AY9" s="10">
-        <f t="shared" si="3"/>
-        <v>75.952466377748195</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AZ9" s="10">
-        <f t="shared" si="3"/>
-        <v>55.038019114309556</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="BA9" s="10">
-        <f t="shared" si="3"/>
-        <v>39.882622546600608</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2174,22 +2215,60 @@
     <row r="30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="33" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="37" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C42">
+        <v>4200</v>
+      </c>
+      <c r="D42">
+        <v>1900</v>
+      </c>
+      <c r="E42">
+        <v>8000</v>
+      </c>
+      <c r="F42">
+        <v>6100</v>
+      </c>
+      <c r="G42">
+        <v>27700</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3328,212 +3407,162 @@
         <v>15</v>
       </c>
       <c r="B2" s="10">
-        <f>'coal retirement'!B3</f>
         <v>0</v>
       </c>
       <c r="C2" s="10">
-        <f>'coal retirement'!C9</f>
         <v>0</v>
       </c>
       <c r="D2" s="10">
-        <f>'coal retirement'!D9</f>
         <v>0</v>
       </c>
       <c r="E2" s="10">
-        <f>'coal retirement'!E9</f>
         <v>0</v>
       </c>
       <c r="F2" s="10">
-        <f>'coal retirement'!F9</f>
         <v>0</v>
       </c>
       <c r="G2" s="10">
-        <f>'coal retirement'!G9</f>
         <v>0</v>
       </c>
       <c r="H2" s="10">
-        <f>'coal retirement'!H9</f>
-        <v>1100</v>
+        <f>'coal retirement'!C42</f>
+        <v>4200</v>
       </c>
       <c r="I2" s="10">
-        <f>'coal retirement'!I9</f>
         <v>0</v>
       </c>
       <c r="J2" s="10">
-        <f>'coal retirement'!J9</f>
         <v>0</v>
       </c>
       <c r="K2" s="10">
-        <f>'coal retirement'!K9</f>
         <v>0</v>
       </c>
       <c r="L2" s="10">
-        <f>'coal retirement'!L9</f>
         <v>0</v>
       </c>
       <c r="M2" s="10">
-        <f>'coal retirement'!M9</f>
-        <v>1000</v>
+        <f>'coal retirement'!D42</f>
+        <v>1900</v>
       </c>
       <c r="N2" s="10">
-        <f>'coal retirement'!N9</f>
         <v>0</v>
       </c>
       <c r="O2" s="10">
-        <f>'coal retirement'!O9</f>
         <v>0</v>
       </c>
       <c r="P2" s="10">
-        <f>'coal retirement'!P9</f>
         <v>0</v>
       </c>
       <c r="Q2" s="10">
-        <f>'coal retirement'!Q9</f>
         <v>0</v>
       </c>
       <c r="R2" s="10">
-        <f>'coal retirement'!R9</f>
         <v>0</v>
       </c>
       <c r="S2" s="10">
-        <f>'coal retirement'!S9</f>
         <v>0</v>
       </c>
       <c r="T2" s="10">
-        <f>'coal retirement'!T9</f>
         <v>0</v>
       </c>
       <c r="U2" s="10">
-        <f>'coal retirement'!U9</f>
         <v>0</v>
       </c>
       <c r="V2" s="10">
-        <f>'coal retirement'!V9</f>
         <v>0</v>
       </c>
       <c r="W2" s="10">
-        <f>'coal retirement'!W9</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="X2" s="10">
-        <f>'coal retirement'!X9</f>
         <v>0</v>
       </c>
       <c r="Y2" s="10">
-        <f>'coal retirement'!Y9</f>
         <v>0</v>
       </c>
       <c r="Z2" s="10">
-        <f>'coal retirement'!Z9</f>
         <v>0</v>
       </c>
       <c r="AA2" s="10">
-        <f>'coal retirement'!AA9</f>
         <v>0</v>
       </c>
       <c r="AB2" s="10">
-        <f>'coal retirement'!AB9</f>
-        <v>24000</v>
+        <v>0</v>
       </c>
       <c r="AC2" s="10">
-        <f>'coal retirement'!AC9</f>
-        <v>22100.000000000364</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="10">
-        <f>'coal retirement'!AD9</f>
-        <v>20200.000000000273</v>
+        <v>0</v>
       </c>
       <c r="AE2" s="10">
-        <f>'coal retirement'!AE9</f>
-        <v>18300.000000000182</v>
+        <v>0</v>
       </c>
       <c r="AF2" s="10">
-        <f>'coal retirement'!AF9</f>
-        <v>16400.000000000091</v>
+        <v>0</v>
       </c>
       <c r="AG2" s="10">
-        <f>'coal retirement'!AG9</f>
-        <v>14500</v>
+        <v>0</v>
       </c>
       <c r="AH2" s="10">
-        <f>'coal retirement'!AH9</f>
-        <v>12600.000000000364</v>
+        <v>0</v>
       </c>
       <c r="AI2" s="10">
-        <f>'coal retirement'!AI9</f>
-        <v>10700.000000000273</v>
+        <v>0</v>
       </c>
       <c r="AJ2" s="10">
-        <f>'coal retirement'!AJ9</f>
-        <v>8800.0000000001819</v>
+        <v>0</v>
       </c>
       <c r="AK2" s="10">
-        <f>'coal retirement'!AK9</f>
-        <v>6900.0000000000909</v>
+        <v>0</v>
       </c>
       <c r="AL2" s="10">
-        <f>'coal retirement'!AL9</f>
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="AM2" s="10">
-        <f>'coal retirement'!AM9</f>
-        <v>3623.1884057970537</v>
+        <v>0</v>
       </c>
       <c r="AN2" s="10">
-        <f>'coal retirement'!AN9</f>
-        <v>2625.498844780439</v>
+        <v>0</v>
       </c>
       <c r="AO2" s="10">
-        <f>'coal retirement'!AO9</f>
-        <v>1902.5353947684089</v>
+        <v>0</v>
       </c>
       <c r="AP2" s="10">
-        <f>'coal retirement'!AP9</f>
-        <v>1378.6488367886841</v>
+        <v>0</v>
       </c>
       <c r="AQ2" s="10">
-        <f>'coal retirement'!AQ9</f>
-        <v>999.02089622367089</v>
+        <v>0</v>
       </c>
       <c r="AR2" s="10">
-        <f>'coal retirement'!AR9</f>
-        <v>723.92818566931714</v>
+        <v>0</v>
       </c>
       <c r="AS2" s="10">
-        <f>'coal retirement'!AS9</f>
-        <v>524.5856417893533</v>
+        <v>0</v>
       </c>
       <c r="AT2" s="10">
-        <f>'coal retirement'!AT9</f>
-        <v>380.13452303575821</v>
+        <v>0</v>
       </c>
       <c r="AU2" s="10">
-        <f>'coal retirement'!AU9</f>
-        <v>275.45979930127044</v>
+        <v>0</v>
       </c>
       <c r="AV2" s="10">
-        <f>'coal retirement'!AV9</f>
-        <v>199.60855021830932</v>
+        <v>0</v>
       </c>
       <c r="AW2" s="10">
-        <f>'coal retirement'!AW9</f>
-        <v>144.64387696978744</v>
+        <v>0</v>
       </c>
       <c r="AX2" s="10">
-        <f>'coal retirement'!AX9</f>
-        <v>104.81440360129388</v>
+        <v>0</v>
       </c>
       <c r="AY2" s="10">
-        <f>'coal retirement'!AY9</f>
-        <v>75.952466377748195</v>
+        <v>0</v>
       </c>
       <c r="AZ2" s="10">
-        <f>'coal retirement'!AZ9</f>
-        <v>55.038019114309556</v>
+        <v>0</v>
       </c>
       <c r="BA2" s="10">
-        <f>'coal retirement'!BA9</f>
-        <v>39.882622546600608</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Tufts elec calibration BCRbQ, BECF, BPMCCS, and MPCbS
</commit_message>
<xml_diff>
--- a/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
+++ b/InputData/elec/BCRbQ/BAU Cap Retirements before Quantization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/elec/BCRbQ/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC1D879-A8BD-6940-95F8-60FD319F4D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D60CC50-7280-3E47-BB25-89FDB285D75B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>BCRbQ BAU Capacity Retirements before Quantization</t>
   </si>
@@ -143,6 +143,27 @@
   </si>
   <si>
     <t>GW to MW</t>
+  </si>
+  <si>
+    <t>coal</t>
+  </si>
+  <si>
+    <t>Capacity retirements (MW)</t>
+  </si>
+  <si>
+    <t>2020-2025</t>
+  </si>
+  <si>
+    <t>2026-2030</t>
+  </si>
+  <si>
+    <t>2031-2035</t>
+  </si>
+  <si>
+    <t>2036-2040</t>
+  </si>
+  <si>
+    <t>2041-2045</t>
   </si>
 </sst>
 </file>
@@ -288,6 +309,50 @@
     </xdr:pic>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>70</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5E7F1FC-B333-8796-9C14-49992B89A1F1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9017000" y="6680200"/>
+          <a:ext cx="9867900" cy="5905500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1803,103 +1868,79 @@
         <v>24</v>
       </c>
       <c r="AC3" s="5">
-        <f t="shared" ref="AC3:AK3" si="0">TREND($AB$7:$AC$7,$AB$6:$AC$6,AC2)</f>
-        <v>22.100000000000364</v>
-      </c>
-      <c r="AD3">
-        <f t="shared" si="0"/>
-        <v>20.200000000000273</v>
-      </c>
-      <c r="AE3">
-        <f t="shared" si="0"/>
-        <v>18.300000000000182</v>
-      </c>
-      <c r="AF3">
-        <f t="shared" si="0"/>
-        <v>16.400000000000091</v>
-      </c>
-      <c r="AG3">
-        <f t="shared" si="0"/>
-        <v>14.5</v>
-      </c>
-      <c r="AH3">
-        <f t="shared" si="0"/>
-        <v>12.600000000000364</v>
-      </c>
-      <c r="AI3">
-        <f t="shared" si="0"/>
-        <v>10.700000000000273</v>
-      </c>
-      <c r="AJ3">
-        <f t="shared" si="0"/>
-        <v>8.8000000000001819</v>
-      </c>
-      <c r="AK3">
-        <f t="shared" si="0"/>
-        <v>6.9000000000000909</v>
+        <v>0</v>
+      </c>
+      <c r="AD3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AJ3" s="5">
+        <v>0</v>
+      </c>
+      <c r="AK3" s="5">
+        <v>0</v>
       </c>
       <c r="AL3" s="5">
         <v>5</v>
       </c>
       <c r="AM3" s="5">
-        <f>(AL3+AL3*$AI$5)</f>
-        <v>3.6231884057970536</v>
+        <v>0</v>
       </c>
       <c r="AN3" s="5">
-        <f t="shared" ref="AN3:BA3" si="1">(AM3+AM3*$AI$5)</f>
-        <v>2.6254988447804388</v>
+        <v>0</v>
       </c>
       <c r="AO3" s="5">
-        <f t="shared" si="1"/>
-        <v>1.9025353947684089</v>
+        <v>0</v>
       </c>
       <c r="AP3" s="5">
-        <f t="shared" si="1"/>
-        <v>1.378648836788684</v>
+        <v>0</v>
       </c>
       <c r="AQ3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.99902089622367085</v>
+        <v>0</v>
       </c>
       <c r="AR3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.72392818566931716</v>
+        <v>0</v>
       </c>
       <c r="AS3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.5245856417893533</v>
+        <v>0</v>
       </c>
       <c r="AT3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.38013452303575823</v>
+        <v>0</v>
       </c>
       <c r="AU3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.27545979930127046</v>
+        <v>0</v>
       </c>
       <c r="AV3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.19960855021830931</v>
+        <v>0</v>
       </c>
       <c r="AW3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.14464387696978745</v>
+        <v>0</v>
       </c>
       <c r="AX3" s="5">
-        <f t="shared" si="1"/>
-        <v>0.10481440360129388</v>
+        <v>0</v>
       </c>
       <c r="AY3" s="5">
-        <f t="shared" si="1"/>
-        <v>7.595246637774819E-2</v>
+        <v>0</v>
       </c>
       <c r="AZ3" s="5">
-        <f t="shared" si="1"/>
-        <v>5.5038019114309555E-2</v>
+        <v>0</v>
       </c>
       <c r="BA3" s="5">
-        <f t="shared" si="1"/>
-        <v>3.9882622546600605E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1916,9 +1957,9 @@
       <c r="AH5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="AI5">
+      <c r="AI5" t="e">
         <f>(AL3-AK3)/AK3</f>
-        <v>-0.27536231884058926</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -1943,212 +1984,212 @@
         <v>12</v>
       </c>
       <c r="B9" s="10">
-        <f t="shared" ref="B9:AB9" si="2">B3*$B$5</f>
+        <f t="shared" ref="B9:AB9" si="0">B3*$B$5</f>
         <v>0</v>
       </c>
       <c r="C9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="D9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="E9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>1100</v>
       </c>
       <c r="I9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="J9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="K9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="M9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>1000</v>
       </c>
       <c r="N9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="P9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Q9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="R9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="S9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="T9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="U9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="V9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="W9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>10000</v>
       </c>
       <c r="X9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Y9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="Z9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AA9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="AB9" s="10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>24000</v>
       </c>
       <c r="AC9" s="10">
-        <f t="shared" ref="AC9:BA9" si="3">AC3*$B$5</f>
-        <v>22100.000000000364</v>
+        <f t="shared" ref="AC9:BA9" si="1">AC3*$B$5</f>
+        <v>0</v>
       </c>
       <c r="AD9" s="10">
-        <f t="shared" si="3"/>
-        <v>20200.000000000273</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AE9" s="10">
-        <f t="shared" si="3"/>
-        <v>18300.000000000182</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AF9" s="10">
-        <f t="shared" si="3"/>
-        <v>16400.000000000091</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AG9" s="10">
-        <f t="shared" si="3"/>
-        <v>14500</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AH9" s="10">
-        <f t="shared" si="3"/>
-        <v>12600.000000000364</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AI9" s="10">
-        <f t="shared" si="3"/>
-        <v>10700.000000000273</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AJ9" s="10">
-        <f t="shared" si="3"/>
-        <v>8800.0000000001819</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AK9" s="10">
-        <f t="shared" si="3"/>
-        <v>6900.0000000000909</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AL9" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="1"/>
         <v>5000</v>
       </c>
       <c r="AM9" s="10">
-        <f t="shared" si="3"/>
-        <v>3623.1884057970537</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AN9" s="10">
-        <f t="shared" si="3"/>
-        <v>2625.498844780439</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AO9" s="10">
-        <f t="shared" si="3"/>
-        <v>1902.5353947684089</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AP9" s="10">
-        <f t="shared" si="3"/>
-        <v>1378.6488367886841</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AQ9" s="10">
-        <f t="shared" si="3"/>
-        <v>999.02089622367089</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AR9" s="10">
-        <f t="shared" si="3"/>
-        <v>723.92818566931714</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AS9" s="10">
-        <f t="shared" si="3"/>
-        <v>524.5856417893533</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AT9" s="10">
-        <f t="shared" si="3"/>
-        <v>380.13452303575821</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AU9" s="10">
-        <f t="shared" si="3"/>
-        <v>275.45979930127044</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AV9" s="10">
-        <f t="shared" si="3"/>
-        <v>199.60855021830932</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AW9" s="10">
-        <f t="shared" si="3"/>
-        <v>144.64387696978744</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AX9" s="10">
-        <f t="shared" si="3"/>
-        <v>104.81440360129388</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AY9" s="10">
-        <f t="shared" si="3"/>
-        <v>75.952466377748195</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="AZ9" s="10">
-        <f t="shared" si="3"/>
-        <v>55.038019114309556</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="BA9" s="10">
-        <f t="shared" si="3"/>
-        <v>39.882622546600608</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2174,22 +2215,60 @@
     <row r="30" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="31" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="32" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="33" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="37" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C42">
+        <v>4200</v>
+      </c>
+      <c r="D42">
+        <v>1900</v>
+      </c>
+      <c r="E42">
+        <v>8000</v>
+      </c>
+      <c r="F42">
+        <v>6100</v>
+      </c>
+      <c r="G42">
+        <v>27700</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3328,212 +3407,162 @@
         <v>15</v>
       </c>
       <c r="B2" s="10">
-        <f>'coal retirement'!B3</f>
         <v>0</v>
       </c>
       <c r="C2" s="10">
-        <f>'coal retirement'!C9</f>
         <v>0</v>
       </c>
       <c r="D2" s="10">
-        <f>'coal retirement'!D9</f>
         <v>0</v>
       </c>
       <c r="E2" s="10">
-        <f>'coal retirement'!E9</f>
         <v>0</v>
       </c>
       <c r="F2" s="10">
-        <f>'coal retirement'!F9</f>
         <v>0</v>
       </c>
       <c r="G2" s="10">
-        <f>'coal retirement'!G9</f>
         <v>0</v>
       </c>
       <c r="H2" s="10">
-        <f>'coal retirement'!H9</f>
-        <v>1100</v>
+        <f>'coal retirement'!C42</f>
+        <v>4200</v>
       </c>
       <c r="I2" s="10">
-        <f>'coal retirement'!I9</f>
         <v>0</v>
       </c>
       <c r="J2" s="10">
-        <f>'coal retirement'!J9</f>
         <v>0</v>
       </c>
       <c r="K2" s="10">
-        <f>'coal retirement'!K9</f>
         <v>0</v>
       </c>
       <c r="L2" s="10">
-        <f>'coal retirement'!L9</f>
         <v>0</v>
       </c>
       <c r="M2" s="10">
-        <f>'coal retirement'!M9</f>
-        <v>1000</v>
+        <f>'coal retirement'!D42</f>
+        <v>1900</v>
       </c>
       <c r="N2" s="10">
-        <f>'coal retirement'!N9</f>
         <v>0</v>
       </c>
       <c r="O2" s="10">
-        <f>'coal retirement'!O9</f>
         <v>0</v>
       </c>
       <c r="P2" s="10">
-        <f>'coal retirement'!P9</f>
         <v>0</v>
       </c>
       <c r="Q2" s="10">
-        <f>'coal retirement'!Q9</f>
         <v>0</v>
       </c>
       <c r="R2" s="10">
-        <f>'coal retirement'!R9</f>
         <v>0</v>
       </c>
       <c r="S2" s="10">
-        <f>'coal retirement'!S9</f>
         <v>0</v>
       </c>
       <c r="T2" s="10">
-        <f>'coal retirement'!T9</f>
         <v>0</v>
       </c>
       <c r="U2" s="10">
-        <f>'coal retirement'!U9</f>
         <v>0</v>
       </c>
       <c r="V2" s="10">
-        <f>'coal retirement'!V9</f>
         <v>0</v>
       </c>
       <c r="W2" s="10">
-        <f>'coal retirement'!W9</f>
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="X2" s="10">
-        <f>'coal retirement'!X9</f>
         <v>0</v>
       </c>
       <c r="Y2" s="10">
-        <f>'coal retirement'!Y9</f>
         <v>0</v>
       </c>
       <c r="Z2" s="10">
-        <f>'coal retirement'!Z9</f>
         <v>0</v>
       </c>
       <c r="AA2" s="10">
-        <f>'coal retirement'!AA9</f>
         <v>0</v>
       </c>
       <c r="AB2" s="10">
-        <f>'coal retirement'!AB9</f>
-        <v>24000</v>
+        <v>0</v>
       </c>
       <c r="AC2" s="10">
-        <f>'coal retirement'!AC9</f>
-        <v>22100.000000000364</v>
+        <v>0</v>
       </c>
       <c r="AD2" s="10">
-        <f>'coal retirement'!AD9</f>
-        <v>20200.000000000273</v>
+        <v>0</v>
       </c>
       <c r="AE2" s="10">
-        <f>'coal retirement'!AE9</f>
-        <v>18300.000000000182</v>
+        <v>0</v>
       </c>
       <c r="AF2" s="10">
-        <f>'coal retirement'!AF9</f>
-        <v>16400.000000000091</v>
+        <v>0</v>
       </c>
       <c r="AG2" s="10">
-        <f>'coal retirement'!AG9</f>
-        <v>14500</v>
+        <v>0</v>
       </c>
       <c r="AH2" s="10">
-        <f>'coal retirement'!AH9</f>
-        <v>12600.000000000364</v>
+        <v>0</v>
       </c>
       <c r="AI2" s="10">
-        <f>'coal retirement'!AI9</f>
-        <v>10700.000000000273</v>
+        <v>0</v>
       </c>
       <c r="AJ2" s="10">
-        <f>'coal retirement'!AJ9</f>
-        <v>8800.0000000001819</v>
+        <v>0</v>
       </c>
       <c r="AK2" s="10">
-        <f>'coal retirement'!AK9</f>
-        <v>6900.0000000000909</v>
+        <v>0</v>
       </c>
       <c r="AL2" s="10">
-        <f>'coal retirement'!AL9</f>
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="AM2" s="10">
-        <f>'coal retirement'!AM9</f>
-        <v>3623.1884057970537</v>
+        <v>0</v>
       </c>
       <c r="AN2" s="10">
-        <f>'coal retirement'!AN9</f>
-        <v>2625.498844780439</v>
+        <v>0</v>
       </c>
       <c r="AO2" s="10">
-        <f>'coal retirement'!AO9</f>
-        <v>1902.5353947684089</v>
+        <v>0</v>
       </c>
       <c r="AP2" s="10">
-        <f>'coal retirement'!AP9</f>
-        <v>1378.6488367886841</v>
+        <v>0</v>
       </c>
       <c r="AQ2" s="10">
-        <f>'coal retirement'!AQ9</f>
-        <v>999.02089622367089</v>
+        <v>0</v>
       </c>
       <c r="AR2" s="10">
-        <f>'coal retirement'!AR9</f>
-        <v>723.92818566931714</v>
+        <v>0</v>
       </c>
       <c r="AS2" s="10">
-        <f>'coal retirement'!AS9</f>
-        <v>524.5856417893533</v>
+        <v>0</v>
       </c>
       <c r="AT2" s="10">
-        <f>'coal retirement'!AT9</f>
-        <v>380.13452303575821</v>
+        <v>0</v>
       </c>
       <c r="AU2" s="10">
-        <f>'coal retirement'!AU9</f>
-        <v>275.45979930127044</v>
+        <v>0</v>
       </c>
       <c r="AV2" s="10">
-        <f>'coal retirement'!AV9</f>
-        <v>199.60855021830932</v>
+        <v>0</v>
       </c>
       <c r="AW2" s="10">
-        <f>'coal retirement'!AW9</f>
-        <v>144.64387696978744</v>
+        <v>0</v>
       </c>
       <c r="AX2" s="10">
-        <f>'coal retirement'!AX9</f>
-        <v>104.81440360129388</v>
+        <v>0</v>
       </c>
       <c r="AY2" s="10">
-        <f>'coal retirement'!AY9</f>
-        <v>75.952466377748195</v>
+        <v>0</v>
       </c>
       <c r="AZ2" s="10">
-        <f>'coal retirement'!AZ9</f>
-        <v>55.038019114309556</v>
+        <v>0</v>
       </c>
       <c r="BA2" s="10">
-        <f>'coal retirement'!BA9</f>
-        <v>39.882622546600608</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>